<commit_message>
Update Excel with full Bidaya product catalog
</commit_message>
<xml_diff>
--- a/data/dashboard-data.xlsx
+++ b/data/dashboard-data.xlsx
@@ -30,6 +30,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -46,7 +47,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,14 +55,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00E6E7EA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,16 +437,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,307 +460,1341 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-Products</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Onboarding &amp; Login</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>KYC, Nafath Verification, Registration</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>MVP-1</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Customer registration and identity verification flow</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Personal Finance (PF)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>End-to-end personal finance application flow</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>New PF, Refinance, Top-Up, Merchant</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>MVP-2</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>End-to-end personal finance application with income verification and offer generation</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>PF After Sales</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Early Settlement, Partial Settlement, Refund, Reschedule</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>MVP-3</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>After-sales services for Personal Finance including settlements and refunds</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>flows/refund-process.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Refinance</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>PF Refinance</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>MVP-2</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Refinancing flow for existing personal finance deals</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Top-Up</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>PF Top-Up</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>MVP-2</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Inprogress</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Top-up financing on existing personal finance deals</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Mortgage (Legacy)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>General Mortgage</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>MVP-4</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Original mortgage product — replaced by Retail Mortgage v2</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Mortgage After Sales</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Settlement, Reschedule</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>MVP-5</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>After-sales services for retail mortgage</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Merchant Finance</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Merchant Finance</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>MVP-6</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Consumer-side merchant finance application flow</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Retail Mortgage</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Mortgage application journey for retail customers</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Off-Plan, Ready Unit, Buy &amp; Lease, REDF Subsidized</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>MVP-7</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Comprehensive mortgage with Off-Plan, Ready Unit sub-products and REDF subsidy support</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SME Onboarding &amp; Login</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Company KYC, Entity Registration</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>MVP-1</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>SME company registration and KYC verification</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Working Capital</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Working Capital Loan</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>MVP-2</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Inprogress</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Working capital finance flow for SME customers</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Working Capital After Sales</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Settlement, Refund</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>MVP-3</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Inprogress</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>After-sales services for working capital including refund flow</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Invoice Financing</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Invoice Discounting, Factoring, With/Without Kafala</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>MVP-4</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Invoice discounting and factoring with Kafala options</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Invoice Finance After Sales</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>MVP-5</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>After-sales for invoice financing products</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Fleet Finance</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Fleet Vehicle Finance</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>MVP-6</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Fleet vehicle financing for SME customers</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Fleet After Sales</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>MVP-6 AS</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>After-sales for fleet finance</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>POS Finance</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Secured POS, Unsecured POS, With/Without Kafala</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>MVP-7</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Point of Sale financing with secured and unsecured options</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>SME Branch Channel</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>WC Branch, Invoice Branch, POS Branch, Mortgage Branch</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>MVP-8</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Inprogress</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Branch channel for all SME products — staff-facing</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>SME Mortgage</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>SME</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CEO prototype - updating on mobile and reflecting on branch</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Lending</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Commercial/Property Mortgage</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>MVP-9</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Invoice Discounting</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>SME commercial and property mortgage — CEO prototype</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>SME Mortgage After Sales</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>SME</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>New flows with Kafala and without Kafala options</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>MVP-9 AS</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>After-sales for SME mortgage</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Public &amp; Private Areas</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>App Shell, Navigation, Dashboard</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>MVP-1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>App structure, public pages, private authenticated areas</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Antifraud</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Fraud Detection, Device Fingerprint</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>MVP-2</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Anti-fraud detection and prevention system</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Freelancer Verification</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Certificate Verification</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>MVP-3</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Freelancer certificate verification flow</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>User Profile - Retail</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Profile Details, Settings</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Retail user profile management and personal details</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>User Profile - SME / Company</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Company Profile, Admin</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>SME user and company profile management</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>SMS, Email, Push, In-App</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Notification management across all channels</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Document Management</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Upload, View, Sign</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Working Capital</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SME</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Working capital finance flow for SME customers</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Inprogress</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>POS Finance</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>SME</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Point of Sale financing with Kafala and without Kafala</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Updating</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Fleet Finance</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Fleet financing journey for retail customers</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Merchant Finance</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Merchant financing application flow</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Refinance</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Refinancing flow - comments added</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Updating</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Document upload, viewing, and e-signature management</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -761,16 +1807,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -811,404 +1857,602 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Refund Process</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>After Sales</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>User requests refund from VA linked to a deal. IBAN selection, fee payment, error handling.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>flows/refund-process.html</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Early Settlement</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>After Sales</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Update flow to match new requirements for automation</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Partial Settlement</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Partial settlement payment flow</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Advanced Payment</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>After Sales</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Update new screens for advanced payment flow</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Reschedule Payment</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>After Sales</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Change installment due dates</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>After Sales - Working Capital</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>After Sales</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Reviewing in progress, adding new refund flow</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>SME Mortgage After Sales</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>After Sales</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>After sales flow for SME mortgage product</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Content Creation (3D Icons + Images)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Create all content for all products. In progress with Majed.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Retail User Profile</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Adding new screens for profile details</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>SME User / Company Profile</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Adding new screens for SME profile and company details</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Branch Features</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>User Profile, cancellation request, loan history</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Freelance Verification</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Freelance certificate verification flow</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Document Management</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Update document management flow</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Transaction History</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Common</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Add empty state screen for transaction history</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Kafala Flow (Invoice)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Invoice discounting with Kafala guarantee</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Kafala Flow (POS)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>POS finance with Kafala guarantee</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>REDF Subsidy Integration</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>REDF subsidy eligibility check for mortgage</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Property Evaluation (Qayim)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Property valuation via Qayim for mortgage</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Updating</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1224,13 +2468,13 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1271,449 +2515,449 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Create all content (3D Icons + Images for all products)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Still in progress with Majed</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>After Sales - PF</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Update new screens for advanced payment, add empty state for transaction history, update Early Settlement, update payments flow, update Document Management</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>SME Mortgage CEO Prototype</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Updating on mobile and to reflect on the branch</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Complete Branch Features</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>User Profile - Cancellation Request - Loan History</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Invoice Discounting</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Add new flow with Kafala and without Kafala</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>After Sales - Working Capital</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>In progress for reviewing, will add new flow for refund</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Inprogress</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Refinance Flow</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Added some comments</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>POS</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Add new flow with Kafala and without Kafala</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Add new form</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Updating</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Retail User Management - Profile Details</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Adding new screens for profile</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>SME User Management - Profile / Company</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Adding new screens for profile</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Mobile</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Retail Mortgage Flow</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Fleet Finance Flow</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Merchant Flow</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>SME Mortgage After Sales Flow</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>After Sales - Working Capital (Branch)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Freelance Verification Flow</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>